<commit_message>
Actualización de mapa con función leaflet para que no se desconecte Shiny. División de mapa por provincias.
</commit_message>
<xml_diff>
--- a/Datos limpios/Pricing diario/2025/Cebada.xlsx
+++ b/Datos limpios/Pricing diario/2025/Cebada.xlsx
@@ -355,7 +355,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K219"/>
+  <dimension ref="A1:K238"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="20.7109375" style="2" customWidth="1"/>
@@ -8452,33 +8452,736 @@
         <v>45957</v>
       </c>
       <c r="B219">
+        <v>7856.26</v>
+      </c>
+      <c r="C219">
+        <v>0</v>
+      </c>
+      <c r="D219">
+        <v>0</v>
+      </c>
+      <c r="E219">
+        <v>7856.26</v>
+      </c>
+      <c r="F219">
+        <v>11532.08</v>
+      </c>
+      <c r="G219">
+        <v>0</v>
+      </c>
+      <c r="H219">
+        <v>0</v>
+      </c>
+      <c r="I219">
+        <v>11532.08</v>
+      </c>
+      <c r="J219">
+        <v>19388.34</v>
+      </c>
+      <c r="K219" t="inlineStr">
+        <is>
+          <t>CEBADA</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" s="2">
+        <v>45958</v>
+      </c>
+      <c r="B220">
+        <v>10205.26</v>
+      </c>
+      <c r="C220">
+        <v>0</v>
+      </c>
+      <c r="D220">
+        <v>0</v>
+      </c>
+      <c r="E220">
+        <v>10205.26</v>
+      </c>
+      <c r="F220">
+        <v>8016</v>
+      </c>
+      <c r="G220">
+        <v>0</v>
+      </c>
+      <c r="H220">
+        <v>0</v>
+      </c>
+      <c r="I220">
+        <v>8016</v>
+      </c>
+      <c r="J220">
+        <v>18221.26</v>
+      </c>
+      <c r="K220" t="inlineStr">
+        <is>
+          <t>CEBADA</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" s="2">
+        <v>45959</v>
+      </c>
+      <c r="B221">
+        <v>10783</v>
+      </c>
+      <c r="C221">
+        <v>1030</v>
+      </c>
+      <c r="D221">
+        <v>340</v>
+      </c>
+      <c r="E221">
+        <v>11473</v>
+      </c>
+      <c r="F221">
+        <v>300</v>
+      </c>
+      <c r="G221">
+        <v>0</v>
+      </c>
+      <c r="H221">
+        <v>0</v>
+      </c>
+      <c r="I221">
+        <v>300</v>
+      </c>
+      <c r="J221">
+        <v>11773</v>
+      </c>
+      <c r="K221" t="inlineStr">
+        <is>
+          <t>CEBADA</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" s="2">
+        <v>45960</v>
+      </c>
+      <c r="B222">
+        <v>18056.23</v>
+      </c>
+      <c r="C222">
+        <v>0</v>
+      </c>
+      <c r="D222">
+        <v>0</v>
+      </c>
+      <c r="E222">
+        <v>18056.23</v>
+      </c>
+      <c r="F222">
+        <v>3480</v>
+      </c>
+      <c r="G222">
+        <v>0</v>
+      </c>
+      <c r="H222">
+        <v>0</v>
+      </c>
+      <c r="I222">
+        <v>3480</v>
+      </c>
+      <c r="J222">
+        <v>21536.23</v>
+      </c>
+      <c r="K222" t="inlineStr">
+        <is>
+          <t>CEBADA</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" s="2">
+        <v>45961</v>
+      </c>
+      <c r="B223">
+        <v>30580</v>
+      </c>
+      <c r="C223">
+        <v>0</v>
+      </c>
+      <c r="D223">
+        <v>150</v>
+      </c>
+      <c r="E223">
+        <v>30430</v>
+      </c>
+      <c r="F223">
+        <v>930</v>
+      </c>
+      <c r="G223">
+        <v>0</v>
+      </c>
+      <c r="H223">
+        <v>0</v>
+      </c>
+      <c r="I223">
+        <v>930</v>
+      </c>
+      <c r="J223">
+        <v>31360</v>
+      </c>
+      <c r="K223" t="inlineStr">
+        <is>
+          <t>CEBADA</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" s="2">
+        <v>45964</v>
+      </c>
+      <c r="B224">
+        <v>26005.8</v>
+      </c>
+      <c r="C224">
+        <v>0</v>
+      </c>
+      <c r="D224">
+        <v>0</v>
+      </c>
+      <c r="E224">
+        <v>26005.8</v>
+      </c>
+      <c r="F224">
         <v>450</v>
       </c>
-      <c r="C219">
-        <v>0</v>
-      </c>
-      <c r="D219">
-        <v>0</v>
-      </c>
-      <c r="E219">
+      <c r="G224">
+        <v>0</v>
+      </c>
+      <c r="H224">
+        <v>0</v>
+      </c>
+      <c r="I224">
         <v>450</v>
       </c>
-      <c r="F219">
-        <v>7500</v>
-      </c>
-      <c r="G219">
-        <v>0</v>
-      </c>
-      <c r="H219">
-        <v>0</v>
-      </c>
-      <c r="I219">
-        <v>7500</v>
-      </c>
-      <c r="J219">
-        <v>7950</v>
-      </c>
-      <c r="K219" t="inlineStr">
+      <c r="J224">
+        <v>26455.8</v>
+      </c>
+      <c r="K224" t="inlineStr">
+        <is>
+          <t>CEBADA</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" s="2">
+        <v>45965</v>
+      </c>
+      <c r="B225">
+        <v>8770</v>
+      </c>
+      <c r="C225">
+        <v>0</v>
+      </c>
+      <c r="D225">
+        <v>0</v>
+      </c>
+      <c r="E225">
+        <v>8770</v>
+      </c>
+      <c r="F225">
+        <v>32590.76</v>
+      </c>
+      <c r="G225">
+        <v>0</v>
+      </c>
+      <c r="H225">
+        <v>0</v>
+      </c>
+      <c r="I225">
+        <v>32590.76</v>
+      </c>
+      <c r="J225">
+        <v>41360.75999999999</v>
+      </c>
+      <c r="K225" t="inlineStr">
+        <is>
+          <t>CEBADA</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" s="2">
+        <v>45966</v>
+      </c>
+      <c r="B226">
+        <v>20645.77</v>
+      </c>
+      <c r="C226">
+        <v>0</v>
+      </c>
+      <c r="D226">
+        <v>0</v>
+      </c>
+      <c r="E226">
+        <v>20645.77</v>
+      </c>
+      <c r="F226">
+        <v>27.88</v>
+      </c>
+      <c r="G226">
+        <v>0</v>
+      </c>
+      <c r="H226">
+        <v>0</v>
+      </c>
+      <c r="I226">
+        <v>27.88</v>
+      </c>
+      <c r="J226">
+        <v>20673.65</v>
+      </c>
+      <c r="K226" t="inlineStr">
+        <is>
+          <t>CEBADA</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" s="2">
+        <v>45967</v>
+      </c>
+      <c r="B227">
+        <v>12972.76</v>
+      </c>
+      <c r="C227">
+        <v>0</v>
+      </c>
+      <c r="D227">
+        <v>2000</v>
+      </c>
+      <c r="E227">
+        <v>10972.76</v>
+      </c>
+      <c r="F227">
+        <v>1320</v>
+      </c>
+      <c r="G227">
+        <v>0</v>
+      </c>
+      <c r="H227">
+        <v>0</v>
+      </c>
+      <c r="I227">
+        <v>1320</v>
+      </c>
+      <c r="J227">
+        <v>12292.76</v>
+      </c>
+      <c r="K227" t="inlineStr">
+        <is>
+          <t>CEBADA</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" s="2">
+        <v>45968</v>
+      </c>
+      <c r="B228">
+        <v>16406.74</v>
+      </c>
+      <c r="C228">
+        <v>0</v>
+      </c>
+      <c r="D228">
+        <v>0</v>
+      </c>
+      <c r="E228">
+        <v>16406.74</v>
+      </c>
+      <c r="F228">
+        <v>7378.32</v>
+      </c>
+      <c r="G228">
+        <v>0</v>
+      </c>
+      <c r="H228">
+        <v>0</v>
+      </c>
+      <c r="I228">
+        <v>7378.32</v>
+      </c>
+      <c r="J228">
+        <v>23785.06</v>
+      </c>
+      <c r="K228" t="inlineStr">
+        <is>
+          <t>CEBADA</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" s="2">
+        <v>45971</v>
+      </c>
+      <c r="B229">
+        <v>14869.99</v>
+      </c>
+      <c r="C229">
+        <v>60</v>
+      </c>
+      <c r="D229">
+        <v>280</v>
+      </c>
+      <c r="E229">
+        <v>14649.99</v>
+      </c>
+      <c r="F229">
+        <v>150</v>
+      </c>
+      <c r="G229">
+        <v>0</v>
+      </c>
+      <c r="H229">
+        <v>0</v>
+      </c>
+      <c r="I229">
+        <v>150</v>
+      </c>
+      <c r="J229">
+        <v>14799.99</v>
+      </c>
+      <c r="K229" t="inlineStr">
+        <is>
+          <t>CEBADA</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" s="2">
+        <v>45972</v>
+      </c>
+      <c r="B230">
+        <v>21980.6</v>
+      </c>
+      <c r="C230">
+        <v>0</v>
+      </c>
+      <c r="D230">
+        <v>0</v>
+      </c>
+      <c r="E230">
+        <v>21980.6</v>
+      </c>
+      <c r="F230">
+        <v>80</v>
+      </c>
+      <c r="G230">
+        <v>0</v>
+      </c>
+      <c r="H230">
+        <v>0</v>
+      </c>
+      <c r="I230">
+        <v>80</v>
+      </c>
+      <c r="J230">
+        <v>22060.6</v>
+      </c>
+      <c r="K230" t="inlineStr">
+        <is>
+          <t>CEBADA</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" s="2">
+        <v>45973</v>
+      </c>
+      <c r="B231">
+        <v>10611.56</v>
+      </c>
+      <c r="C231">
+        <v>0</v>
+      </c>
+      <c r="D231">
+        <v>130</v>
+      </c>
+      <c r="E231">
+        <v>10481.56</v>
+      </c>
+      <c r="F231">
+        <v>0</v>
+      </c>
+      <c r="G231">
+        <v>0</v>
+      </c>
+      <c r="H231">
+        <v>0</v>
+      </c>
+      <c r="I231">
+        <v>0</v>
+      </c>
+      <c r="J231">
+        <v>10481.56</v>
+      </c>
+      <c r="K231" t="inlineStr">
+        <is>
+          <t>CEBADA</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" s="2">
+        <v>45974</v>
+      </c>
+      <c r="B232">
+        <v>15739.25</v>
+      </c>
+      <c r="C232">
+        <v>0</v>
+      </c>
+      <c r="D232">
+        <v>0</v>
+      </c>
+      <c r="E232">
+        <v>15739.25</v>
+      </c>
+      <c r="F232">
+        <v>0</v>
+      </c>
+      <c r="G232">
+        <v>0</v>
+      </c>
+      <c r="H232">
+        <v>0</v>
+      </c>
+      <c r="I232">
+        <v>0</v>
+      </c>
+      <c r="J232">
+        <v>15739.25</v>
+      </c>
+      <c r="K232" t="inlineStr">
+        <is>
+          <t>CEBADA</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" s="2">
+        <v>45975</v>
+      </c>
+      <c r="B233">
+        <v>12582.57</v>
+      </c>
+      <c r="C233">
+        <v>2000</v>
+      </c>
+      <c r="D233">
+        <v>0</v>
+      </c>
+      <c r="E233">
+        <v>14582.57</v>
+      </c>
+      <c r="F233">
+        <v>40</v>
+      </c>
+      <c r="G233">
+        <v>0</v>
+      </c>
+      <c r="H233">
+        <v>0</v>
+      </c>
+      <c r="I233">
+        <v>40</v>
+      </c>
+      <c r="J233">
+        <v>14622.57</v>
+      </c>
+      <c r="K233" t="inlineStr">
+        <is>
+          <t>CEBADA</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" s="2">
+        <v>45978</v>
+      </c>
+      <c r="B234">
+        <v>17610.74</v>
+      </c>
+      <c r="C234">
+        <v>0</v>
+      </c>
+      <c r="D234">
+        <v>60</v>
+      </c>
+      <c r="E234">
+        <v>17550.74</v>
+      </c>
+      <c r="F234">
+        <v>14198</v>
+      </c>
+      <c r="G234">
+        <v>0</v>
+      </c>
+      <c r="H234">
+        <v>0</v>
+      </c>
+      <c r="I234">
+        <v>14198</v>
+      </c>
+      <c r="J234">
+        <v>31748.74</v>
+      </c>
+      <c r="K234" t="inlineStr">
+        <is>
+          <t>CEBADA</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" s="2">
+        <v>45979</v>
+      </c>
+      <c r="B235">
+        <v>28003.37</v>
+      </c>
+      <c r="C235">
+        <v>0</v>
+      </c>
+      <c r="D235">
+        <v>1000</v>
+      </c>
+      <c r="E235">
+        <v>27003.37</v>
+      </c>
+      <c r="F235">
+        <v>420</v>
+      </c>
+      <c r="G235">
+        <v>0</v>
+      </c>
+      <c r="H235">
+        <v>0</v>
+      </c>
+      <c r="I235">
+        <v>420</v>
+      </c>
+      <c r="J235">
+        <v>27423.37</v>
+      </c>
+      <c r="K235" t="inlineStr">
+        <is>
+          <t>CEBADA</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" s="2">
+        <v>45980</v>
+      </c>
+      <c r="B236">
+        <v>25271</v>
+      </c>
+      <c r="C236">
+        <v>0</v>
+      </c>
+      <c r="D236">
+        <v>0</v>
+      </c>
+      <c r="E236">
+        <v>25271</v>
+      </c>
+      <c r="F236">
+        <v>1785</v>
+      </c>
+      <c r="G236">
+        <v>0</v>
+      </c>
+      <c r="H236">
+        <v>0</v>
+      </c>
+      <c r="I236">
+        <v>1785</v>
+      </c>
+      <c r="J236">
+        <v>27056</v>
+      </c>
+      <c r="K236" t="inlineStr">
+        <is>
+          <t>CEBADA</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" s="2">
+        <v>45981</v>
+      </c>
+      <c r="B237">
+        <v>26505.74</v>
+      </c>
+      <c r="C237">
+        <v>2200</v>
+      </c>
+      <c r="D237">
+        <v>300</v>
+      </c>
+      <c r="E237">
+        <v>28405.74</v>
+      </c>
+      <c r="F237">
+        <v>1010</v>
+      </c>
+      <c r="G237">
+        <v>0</v>
+      </c>
+      <c r="H237">
+        <v>0</v>
+      </c>
+      <c r="I237">
+        <v>1010</v>
+      </c>
+      <c r="J237">
+        <v>29415.74</v>
+      </c>
+      <c r="K237" t="inlineStr">
+        <is>
+          <t>CEBADA</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" s="2">
+        <v>45982</v>
+      </c>
+      <c r="B238">
+        <v>10210</v>
+      </c>
+      <c r="C238">
+        <v>0</v>
+      </c>
+      <c r="D238">
+        <v>0</v>
+      </c>
+      <c r="E238">
+        <v>10210</v>
+      </c>
+      <c r="F238">
+        <v>0</v>
+      </c>
+      <c r="G238">
+        <v>0</v>
+      </c>
+      <c r="H238">
+        <v>0</v>
+      </c>
+      <c r="I238">
+        <v>0</v>
+      </c>
+      <c r="J238">
+        <v>10210</v>
+      </c>
+      <c r="K238" t="inlineStr">
         <is>
           <t>CEBADA</t>
         </is>

</xml_diff>